<commit_message>
Fix AP Macro/Micro (765/766) to Semester/2.5 credits
Per principal's correction: both courses are semester-length with 2.5
credits, not full-year/5 as listed in the sectioning template.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/DonBosco_CourseList_2026-27.xlsx
+++ b/DonBosco_CourseList_2026-27.xlsx
@@ -3940,53 +3940,53 @@
       </c>
     </row>
     <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="7" t="inlineStr">
+      <c r="A144" s="4" t="inlineStr">
         <is>
           <t>765</t>
         </is>
       </c>
-      <c r="B144" s="8" t="inlineStr">
+      <c r="B144" s="5" t="inlineStr">
         <is>
           <t>AP Macroeconomics</t>
         </is>
       </c>
-      <c r="C144" s="8" t="inlineStr">
+      <c r="C144" s="5" t="inlineStr">
         <is>
           <t>Social Studies</t>
         </is>
       </c>
-      <c r="D144" s="9" t="inlineStr">
-        <is>
-          <t>FY</t>
-        </is>
-      </c>
-      <c r="E144" s="9" t="n">
-        <v>5</v>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>SEM</t>
+        </is>
+      </c>
+      <c r="E144" s="6" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="145" ht="18" customHeight="1">
-      <c r="A145" s="7" t="inlineStr">
+      <c r="A145" s="4" t="inlineStr">
         <is>
           <t>766</t>
         </is>
       </c>
-      <c r="B145" s="8" t="inlineStr">
+      <c r="B145" s="5" t="inlineStr">
         <is>
           <t>AP Microeconomics</t>
         </is>
       </c>
-      <c r="C145" s="8" t="inlineStr">
+      <c r="C145" s="5" t="inlineStr">
         <is>
           <t>Social Studies</t>
         </is>
       </c>
-      <c r="D145" s="9" t="inlineStr">
-        <is>
-          <t>FY</t>
-        </is>
-      </c>
-      <c r="E145" s="9" t="n">
-        <v>5</v>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>SEM</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="146" ht="22" customHeight="1">
@@ -4242,7 +4242,7 @@
         </is>
       </c>
       <c r="B159" s="10" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C159" s="11" t="n"/>
       <c r="D159" s="11" t="n"/>
@@ -4255,7 +4255,7 @@
         </is>
       </c>
       <c r="B160" s="10" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C160" s="11" t="n"/>
       <c r="D160" s="11" t="n"/>

</xml_diff>